<commit_message>
principal component analysis on several datasets
</commit_message>
<xml_diff>
--- a/PCA_datasets.xlsx
+++ b/PCA_datasets.xlsx
@@ -8,25 +8,36 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5ee7d9eaf30fc32d/Documents/CSE_4205/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_DAD177870A09E956244D81567F55A2E0CA540F7D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F01ED8E4-CA3E-4C51-9971-42B5EB4CEFB8}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{752BD980-A988-46B7-A3AE-29E79F0436EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Foods" sheetId="1" r:id="rId1"/>
     <sheet name="Cars" sheetId="2" r:id="rId2"/>
     <sheet name="Students" sheetId="3" r:id="rId3"/>
     <sheet name="Cities" sheetId="4" r:id="rId4"/>
+    <sheet name="Students_scores" sheetId="7" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="67">
-  <si>
-    <t>Product</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="161">
   <si>
     <t>Protein_g</t>
   </si>
@@ -224,6 +235,291 @@
   </si>
   <si>
     <t>Atlanta</t>
+  </si>
+  <si>
+    <t>Math_Score</t>
+  </si>
+  <si>
+    <t>Physics_Score</t>
+  </si>
+  <si>
+    <t>Literature_Score</t>
+  </si>
+  <si>
+    <t>History_Score</t>
+  </si>
+  <si>
+    <t>Shoe_Size_EU</t>
+  </si>
+  <si>
+    <t>S13</t>
+  </si>
+  <si>
+    <t>S14</t>
+  </si>
+  <si>
+    <t>S15</t>
+  </si>
+  <si>
+    <t>S16</t>
+  </si>
+  <si>
+    <t>S17</t>
+  </si>
+  <si>
+    <t>S18</t>
+  </si>
+  <si>
+    <t>S19</t>
+  </si>
+  <si>
+    <t>S20</t>
+  </si>
+  <si>
+    <t>S21</t>
+  </si>
+  <si>
+    <t>S22</t>
+  </si>
+  <si>
+    <t>S23</t>
+  </si>
+  <si>
+    <t>S24</t>
+  </si>
+  <si>
+    <t>S25</t>
+  </si>
+  <si>
+    <t>S26</t>
+  </si>
+  <si>
+    <t>S27</t>
+  </si>
+  <si>
+    <t>S28</t>
+  </si>
+  <si>
+    <t>S29</t>
+  </si>
+  <si>
+    <t>S30</t>
+  </si>
+  <si>
+    <t>S31</t>
+  </si>
+  <si>
+    <t>S32</t>
+  </si>
+  <si>
+    <t>S33</t>
+  </si>
+  <si>
+    <t>S34</t>
+  </si>
+  <si>
+    <t>S35</t>
+  </si>
+  <si>
+    <t>S36</t>
+  </si>
+  <si>
+    <t>S37</t>
+  </si>
+  <si>
+    <t>S38</t>
+  </si>
+  <si>
+    <t>S39</t>
+  </si>
+  <si>
+    <t>S40</t>
+  </si>
+  <si>
+    <t>S41</t>
+  </si>
+  <si>
+    <t>S42</t>
+  </si>
+  <si>
+    <t>S43</t>
+  </si>
+  <si>
+    <t>S44</t>
+  </si>
+  <si>
+    <t>S45</t>
+  </si>
+  <si>
+    <t>S46</t>
+  </si>
+  <si>
+    <t>S47</t>
+  </si>
+  <si>
+    <t>S48</t>
+  </si>
+  <si>
+    <t>S49</t>
+  </si>
+  <si>
+    <t>S50</t>
+  </si>
+  <si>
+    <t>S51</t>
+  </si>
+  <si>
+    <t>S52</t>
+  </si>
+  <si>
+    <t>S53</t>
+  </si>
+  <si>
+    <t>S54</t>
+  </si>
+  <si>
+    <t>S55</t>
+  </si>
+  <si>
+    <t>S56</t>
+  </si>
+  <si>
+    <t>S57</t>
+  </si>
+  <si>
+    <t>S58</t>
+  </si>
+  <si>
+    <t>S59</t>
+  </si>
+  <si>
+    <t>S60</t>
+  </si>
+  <si>
+    <t>S61</t>
+  </si>
+  <si>
+    <t>S62</t>
+  </si>
+  <si>
+    <t>S63</t>
+  </si>
+  <si>
+    <t>S64</t>
+  </si>
+  <si>
+    <t>S65</t>
+  </si>
+  <si>
+    <t>S66</t>
+  </si>
+  <si>
+    <t>S67</t>
+  </si>
+  <si>
+    <t>S68</t>
+  </si>
+  <si>
+    <t>S69</t>
+  </si>
+  <si>
+    <t>S70</t>
+  </si>
+  <si>
+    <t>S71</t>
+  </si>
+  <si>
+    <t>S72</t>
+  </si>
+  <si>
+    <t>S73</t>
+  </si>
+  <si>
+    <t>S74</t>
+  </si>
+  <si>
+    <t>S75</t>
+  </si>
+  <si>
+    <t>S76</t>
+  </si>
+  <si>
+    <t>S77</t>
+  </si>
+  <si>
+    <t>S78</t>
+  </si>
+  <si>
+    <t>S79</t>
+  </si>
+  <si>
+    <t>S80</t>
+  </si>
+  <si>
+    <t>S81</t>
+  </si>
+  <si>
+    <t>S82</t>
+  </si>
+  <si>
+    <t>S83</t>
+  </si>
+  <si>
+    <t>S84</t>
+  </si>
+  <si>
+    <t>S85</t>
+  </si>
+  <si>
+    <t>S86</t>
+  </si>
+  <si>
+    <t>S87</t>
+  </si>
+  <si>
+    <t>S88</t>
+  </si>
+  <si>
+    <t>S89</t>
+  </si>
+  <si>
+    <t>S90</t>
+  </si>
+  <si>
+    <t>S91</t>
+  </si>
+  <si>
+    <t>S92</t>
+  </si>
+  <si>
+    <t>S93</t>
+  </si>
+  <si>
+    <t>S94</t>
+  </si>
+  <si>
+    <t>S95</t>
+  </si>
+  <si>
+    <t>S96</t>
+  </si>
+  <si>
+    <t>S97</t>
+  </si>
+  <si>
+    <t>S98</t>
+  </si>
+  <si>
+    <t>S99</t>
+  </si>
+  <si>
+    <t>S100</t>
+  </si>
+  <si>
+    <t>Students_scores</t>
+  </si>
+  <si>
+    <t>Foods</t>
   </si>
 </sst>
 </file>
@@ -584,24 +880,24 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B2" s="2">
         <v>3.2</v>
@@ -618,7 +914,7 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B3" s="2">
         <v>4</v>
@@ -635,7 +931,7 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B4" s="2">
         <v>25</v>
@@ -652,7 +948,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B5" s="2">
         <v>9</v>
@@ -669,7 +965,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B6" s="2">
         <v>2.7</v>
@@ -686,7 +982,7 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B7" s="2">
         <v>0.3</v>
@@ -703,7 +999,7 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B8" s="2">
         <v>1.3</v>
@@ -720,7 +1016,7 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B9" s="2">
         <v>27</v>
@@ -737,7 +1033,7 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B10" s="2">
         <v>20</v>
@@ -754,7 +1050,7 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B11" s="2">
         <v>13</v>
@@ -787,27 +1083,27 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>19</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B2" s="2">
         <v>27000</v>
@@ -827,7 +1123,7 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B3" s="2">
         <v>28000</v>
@@ -847,7 +1143,7 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B4" s="2">
         <v>35000</v>
@@ -867,7 +1163,7 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B5" s="2">
         <v>52000</v>
@@ -887,7 +1183,7 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B6" s="2">
         <v>48000</v>
@@ -907,7 +1203,7 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B7" s="2">
         <v>30000</v>
@@ -927,7 +1223,7 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B8" s="2">
         <v>38000</v>
@@ -947,7 +1243,7 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B9" s="2">
         <v>95000</v>
@@ -967,7 +1263,7 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B10" s="2">
         <v>29000</v>
@@ -987,7 +1283,7 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B11" s="2">
         <v>34000</v>
@@ -1022,27 +1318,27 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>35</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B2" s="2">
         <v>92</v>
@@ -1062,7 +1358,7 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B3" s="2">
         <v>88</v>
@@ -1082,7 +1378,7 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B4" s="2">
         <v>75</v>
@@ -1102,7 +1398,7 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B5" s="2">
         <v>70</v>
@@ -1122,7 +1418,7 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B6" s="2">
         <v>95</v>
@@ -1142,7 +1438,7 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B7" s="2">
         <v>65</v>
@@ -1162,7 +1458,7 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B8" s="2">
         <v>84</v>
@@ -1182,7 +1478,7 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B9" s="2">
         <v>78</v>
@@ -1202,7 +1498,7 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B10" s="2">
         <v>60</v>
@@ -1222,7 +1518,7 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B11" s="2">
         <v>91</v>
@@ -1242,7 +1538,7 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B12" s="2">
         <v>73</v>
@@ -1262,7 +1558,7 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B13" s="2">
         <v>82</v>
@@ -1298,27 +1594,27 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>53</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B2" s="2">
         <v>63</v>
@@ -1338,7 +1634,7 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B3" s="2">
         <v>55</v>
@@ -1358,7 +1654,7 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B4" s="2">
         <v>51</v>
@@ -1378,7 +1674,7 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B5" s="2">
         <v>53</v>
@@ -1398,7 +1694,7 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B6" s="2">
         <v>77</v>
@@ -1418,7 +1714,7 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B7" s="2">
         <v>50</v>
@@ -1438,7 +1734,7 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B8" s="2">
         <v>67</v>
@@ -1458,7 +1754,7 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B9" s="2">
         <v>75</v>
@@ -1478,7 +1774,7 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B10" s="2">
         <v>60</v>
@@ -1498,7 +1794,7 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B11" s="2">
         <v>66</v>
@@ -1518,7 +1814,7 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B12" s="2">
         <v>54</v>
@@ -1538,7 +1834,7 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B13" s="2">
         <v>68</v>
@@ -1559,4 +1855,2034 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DCBD6CC8-AFA2-4A4C-8DAD-298BE9EC38D7}">
+  <dimension ref="A1:F101"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>159</v>
+      </c>
+      <c r="B1" t="s">
+        <v>66</v>
+      </c>
+      <c r="C1" t="s">
+        <v>67</v>
+      </c>
+      <c r="D1" t="s">
+        <v>68</v>
+      </c>
+      <c r="E1" t="s">
+        <v>69</v>
+      </c>
+      <c r="F1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B2">
+        <v>75.400000000000006</v>
+      </c>
+      <c r="C2">
+        <v>72.7</v>
+      </c>
+      <c r="D2">
+        <v>80.5</v>
+      </c>
+      <c r="E2">
+        <v>80.400000000000006</v>
+      </c>
+      <c r="F2">
+        <v>38.700000000000003</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B3">
+        <v>74.8</v>
+      </c>
+      <c r="C3">
+        <v>75.3</v>
+      </c>
+      <c r="D3">
+        <v>79.099999999999994</v>
+      </c>
+      <c r="E3">
+        <v>68.2</v>
+      </c>
+      <c r="F3">
+        <v>42.6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>38</v>
+      </c>
+      <c r="B4">
+        <v>87</v>
+      </c>
+      <c r="C4">
+        <v>85.4</v>
+      </c>
+      <c r="D4">
+        <v>76.3</v>
+      </c>
+      <c r="E4">
+        <v>85.3</v>
+      </c>
+      <c r="F4">
+        <v>38.200000000000003</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>39</v>
+      </c>
+      <c r="B5">
+        <v>93.1</v>
+      </c>
+      <c r="C5">
+        <v>91.6</v>
+      </c>
+      <c r="D5">
+        <v>92.8</v>
+      </c>
+      <c r="E5">
+        <v>95.9</v>
+      </c>
+      <c r="F5">
+        <v>36.5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>40</v>
+      </c>
+      <c r="B6">
+        <v>76.8</v>
+      </c>
+      <c r="C6">
+        <v>76.3</v>
+      </c>
+      <c r="D6">
+        <v>58.2</v>
+      </c>
+      <c r="E6">
+        <v>64.8</v>
+      </c>
+      <c r="F6">
+        <v>36.1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>41</v>
+      </c>
+      <c r="B7">
+        <v>80</v>
+      </c>
+      <c r="C7">
+        <v>83</v>
+      </c>
+      <c r="D7">
+        <v>61</v>
+      </c>
+      <c r="E7">
+        <v>72.400000000000006</v>
+      </c>
+      <c r="F7">
+        <v>41.5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>42</v>
+      </c>
+      <c r="B8">
+        <v>100</v>
+      </c>
+      <c r="C8">
+        <v>100</v>
+      </c>
+      <c r="D8">
+        <v>86</v>
+      </c>
+      <c r="E8">
+        <v>85.8</v>
+      </c>
+      <c r="F8">
+        <v>36.799999999999997</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>43</v>
+      </c>
+      <c r="B9">
+        <v>86.8</v>
+      </c>
+      <c r="C9">
+        <v>89.3</v>
+      </c>
+      <c r="D9">
+        <v>76.8</v>
+      </c>
+      <c r="E9">
+        <v>75.8</v>
+      </c>
+      <c r="F9">
+        <v>44.4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>44</v>
+      </c>
+      <c r="B10">
+        <v>78.2</v>
+      </c>
+      <c r="C10">
+        <v>78.2</v>
+      </c>
+      <c r="D10">
+        <v>68.099999999999994</v>
+      </c>
+      <c r="E10">
+        <v>61.3</v>
+      </c>
+      <c r="F10">
+        <v>34.799999999999997</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>45</v>
+      </c>
+      <c r="B11">
+        <v>84.4</v>
+      </c>
+      <c r="C11">
+        <v>87.5</v>
+      </c>
+      <c r="D11">
+        <v>91.4</v>
+      </c>
+      <c r="E11">
+        <v>97.8</v>
+      </c>
+      <c r="F11">
+        <v>44.2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>46</v>
+      </c>
+      <c r="B12">
+        <v>65.099999999999994</v>
+      </c>
+      <c r="C12">
+        <v>67</v>
+      </c>
+      <c r="D12">
+        <v>69.3</v>
+      </c>
+      <c r="E12">
+        <v>71.3</v>
+      </c>
+      <c r="F12">
+        <v>40.5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>47</v>
+      </c>
+      <c r="B13">
+        <v>78.5</v>
+      </c>
+      <c r="C13">
+        <v>72.8</v>
+      </c>
+      <c r="D13">
+        <v>70.8</v>
+      </c>
+      <c r="E13">
+        <v>70.7</v>
+      </c>
+      <c r="F13">
+        <v>39.799999999999997</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>71</v>
+      </c>
+      <c r="B14">
+        <v>85.2</v>
+      </c>
+      <c r="C14">
+        <v>79.2</v>
+      </c>
+      <c r="D14">
+        <v>76.2</v>
+      </c>
+      <c r="E14">
+        <v>78.400000000000006</v>
+      </c>
+      <c r="F14">
+        <v>38.6</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>72</v>
+      </c>
+      <c r="B15">
+        <v>75.599999999999994</v>
+      </c>
+      <c r="C15">
+        <v>80.5</v>
+      </c>
+      <c r="D15">
+        <v>50.5</v>
+      </c>
+      <c r="E15">
+        <v>50</v>
+      </c>
+      <c r="F15">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>73</v>
+      </c>
+      <c r="B16">
+        <v>66.3</v>
+      </c>
+      <c r="C16">
+        <v>63.1</v>
+      </c>
+      <c r="D16">
+        <v>70.099999999999994</v>
+      </c>
+      <c r="E16">
+        <v>67.599999999999994</v>
+      </c>
+      <c r="F16">
+        <v>38.6</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>74</v>
+      </c>
+      <c r="B17">
+        <v>78.8</v>
+      </c>
+      <c r="C17">
+        <v>74.599999999999994</v>
+      </c>
+      <c r="D17">
+        <v>81.599999999999994</v>
+      </c>
+      <c r="E17">
+        <v>79.2</v>
+      </c>
+      <c r="F17">
+        <v>38.6</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>75</v>
+      </c>
+      <c r="B18">
+        <v>59.7</v>
+      </c>
+      <c r="C18">
+        <v>58.2</v>
+      </c>
+      <c r="D18">
+        <v>60</v>
+      </c>
+      <c r="E18">
+        <v>63.8</v>
+      </c>
+      <c r="F18">
+        <v>32.200000000000003</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>76</v>
+      </c>
+      <c r="B19">
+        <v>64.900000000000006</v>
+      </c>
+      <c r="C19">
+        <v>67.7</v>
+      </c>
+      <c r="D19">
+        <v>78.7</v>
+      </c>
+      <c r="E19">
+        <v>78</v>
+      </c>
+      <c r="F19">
+        <v>42.5</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>77</v>
+      </c>
+      <c r="B20">
+        <v>72</v>
+      </c>
+      <c r="C20">
+        <v>74.7</v>
+      </c>
+      <c r="D20">
+        <v>81.099999999999994</v>
+      </c>
+      <c r="E20">
+        <v>84.7</v>
+      </c>
+      <c r="F20">
+        <v>37.700000000000003</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>78</v>
+      </c>
+      <c r="B21">
+        <v>69.3</v>
+      </c>
+      <c r="C21">
+        <v>68.599999999999994</v>
+      </c>
+      <c r="D21">
+        <v>76.099999999999994</v>
+      </c>
+      <c r="E21">
+        <v>75</v>
+      </c>
+      <c r="F21">
+        <v>43.7</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>79</v>
+      </c>
+      <c r="B22">
+        <v>74.099999999999994</v>
+      </c>
+      <c r="C22">
+        <v>76.400000000000006</v>
+      </c>
+      <c r="D22">
+        <v>76.7</v>
+      </c>
+      <c r="E22">
+        <v>72</v>
+      </c>
+      <c r="F22">
+        <v>43.7</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>80</v>
+      </c>
+      <c r="B23">
+        <v>69.7</v>
+      </c>
+      <c r="C23">
+        <v>67.2</v>
+      </c>
+      <c r="D23">
+        <v>75.2</v>
+      </c>
+      <c r="E23">
+        <v>72.900000000000006</v>
+      </c>
+      <c r="F23">
+        <v>40.200000000000003</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>81</v>
+      </c>
+      <c r="B24">
+        <v>78.7</v>
+      </c>
+      <c r="C24">
+        <v>76.2</v>
+      </c>
+      <c r="D24">
+        <v>77.099999999999994</v>
+      </c>
+      <c r="E24">
+        <v>73.7</v>
+      </c>
+      <c r="F24">
+        <v>40.200000000000003</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>82</v>
+      </c>
+      <c r="B25">
+        <v>80.7</v>
+      </c>
+      <c r="C25">
+        <v>82.5</v>
+      </c>
+      <c r="D25">
+        <v>70.8</v>
+      </c>
+      <c r="E25">
+        <v>75.8</v>
+      </c>
+      <c r="F25">
+        <v>34.299999999999997</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>83</v>
+      </c>
+      <c r="B26">
+        <v>72.7</v>
+      </c>
+      <c r="C26">
+        <v>69.400000000000006</v>
+      </c>
+      <c r="D26">
+        <v>78.3</v>
+      </c>
+      <c r="E26">
+        <v>82.7</v>
+      </c>
+      <c r="F26">
+        <v>38.700000000000003</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>84</v>
+      </c>
+      <c r="B27">
+        <v>68.7</v>
+      </c>
+      <c r="C27">
+        <v>71.2</v>
+      </c>
+      <c r="D27">
+        <v>59.9</v>
+      </c>
+      <c r="E27">
+        <v>64.8</v>
+      </c>
+      <c r="F27">
+        <v>41.4</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>85</v>
+      </c>
+      <c r="B28">
+        <v>70.099999999999994</v>
+      </c>
+      <c r="C28">
+        <v>63.8</v>
+      </c>
+      <c r="D28">
+        <v>77.900000000000006</v>
+      </c>
+      <c r="E28">
+        <v>74.900000000000006</v>
+      </c>
+      <c r="F28">
+        <v>37.4</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>86</v>
+      </c>
+      <c r="B29">
+        <v>78.599999999999994</v>
+      </c>
+      <c r="C29">
+        <v>74.900000000000006</v>
+      </c>
+      <c r="D29">
+        <v>91</v>
+      </c>
+      <c r="E29">
+        <v>90.4</v>
+      </c>
+      <c r="F29">
+        <v>39.200000000000003</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>87</v>
+      </c>
+      <c r="B30">
+        <v>74.900000000000006</v>
+      </c>
+      <c r="C30">
+        <v>74.8</v>
+      </c>
+      <c r="D30">
+        <v>69.5</v>
+      </c>
+      <c r="E30">
+        <v>68</v>
+      </c>
+      <c r="F30">
+        <v>38.5</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>88</v>
+      </c>
+      <c r="B31">
+        <v>72.8</v>
+      </c>
+      <c r="C31">
+        <v>76.2</v>
+      </c>
+      <c r="D31">
+        <v>70.8</v>
+      </c>
+      <c r="E31">
+        <v>75.5</v>
+      </c>
+      <c r="F31">
+        <v>39.299999999999997</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>89</v>
+      </c>
+      <c r="B32">
+        <v>67.900000000000006</v>
+      </c>
+      <c r="C32">
+        <v>64.400000000000006</v>
+      </c>
+      <c r="D32">
+        <v>58</v>
+      </c>
+      <c r="E32">
+        <v>55.3</v>
+      </c>
+      <c r="F32">
+        <v>38.5</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>90</v>
+      </c>
+      <c r="B33">
+        <v>87.9</v>
+      </c>
+      <c r="C33">
+        <v>89.7</v>
+      </c>
+      <c r="D33">
+        <v>75.7</v>
+      </c>
+      <c r="E33">
+        <v>80.2</v>
+      </c>
+      <c r="F33">
+        <v>39.799999999999997</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>91</v>
+      </c>
+      <c r="B34">
+        <v>75.8</v>
+      </c>
+      <c r="C34">
+        <v>72.099999999999994</v>
+      </c>
+      <c r="D34">
+        <v>88.1</v>
+      </c>
+      <c r="E34">
+        <v>87.7</v>
+      </c>
+      <c r="F34">
+        <v>39.5</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>92</v>
+      </c>
+      <c r="B35">
+        <v>88.3</v>
+      </c>
+      <c r="C35">
+        <v>84.8</v>
+      </c>
+      <c r="D35">
+        <v>76.5</v>
+      </c>
+      <c r="E35">
+        <v>80.900000000000006</v>
+      </c>
+      <c r="F35">
+        <v>38.299999999999997</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>93</v>
+      </c>
+      <c r="B36">
+        <v>76.5</v>
+      </c>
+      <c r="C36">
+        <v>77.7</v>
+      </c>
+      <c r="D36">
+        <v>71.8</v>
+      </c>
+      <c r="E36">
+        <v>71.5</v>
+      </c>
+      <c r="F36">
+        <v>37.4</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>94</v>
+      </c>
+      <c r="B37">
+        <v>80.3</v>
+      </c>
+      <c r="C37">
+        <v>76.5</v>
+      </c>
+      <c r="D37">
+        <v>71.7</v>
+      </c>
+      <c r="E37">
+        <v>75.099999999999994</v>
+      </c>
+      <c r="F37">
+        <v>34.799999999999997</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>95</v>
+      </c>
+      <c r="B38">
+        <v>73.7</v>
+      </c>
+      <c r="C38">
+        <v>74.599999999999994</v>
+      </c>
+      <c r="D38">
+        <v>75</v>
+      </c>
+      <c r="E38">
+        <v>70.5</v>
+      </c>
+      <c r="F38">
+        <v>39.5</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
+        <v>96</v>
+      </c>
+      <c r="B39">
+        <v>80.5</v>
+      </c>
+      <c r="C39">
+        <v>79.8</v>
+      </c>
+      <c r="D39">
+        <v>69.599999999999994</v>
+      </c>
+      <c r="E39">
+        <v>70.400000000000006</v>
+      </c>
+      <c r="F39">
+        <v>36.6</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>97</v>
+      </c>
+      <c r="B40">
+        <v>70.5</v>
+      </c>
+      <c r="C40">
+        <v>67.099999999999994</v>
+      </c>
+      <c r="D40">
+        <v>81.8</v>
+      </c>
+      <c r="E40">
+        <v>77.900000000000006</v>
+      </c>
+      <c r="F40">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>98</v>
+      </c>
+      <c r="B41">
+        <v>87.4</v>
+      </c>
+      <c r="C41">
+        <v>87.8</v>
+      </c>
+      <c r="D41">
+        <v>71</v>
+      </c>
+      <c r="E41">
+        <v>78.8</v>
+      </c>
+      <c r="F41">
+        <v>38.200000000000003</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
+        <v>99</v>
+      </c>
+      <c r="B42">
+        <v>88</v>
+      </c>
+      <c r="C42">
+        <v>88.2</v>
+      </c>
+      <c r="D42">
+        <v>81.3</v>
+      </c>
+      <c r="E42">
+        <v>86.1</v>
+      </c>
+      <c r="F42">
+        <v>39.5</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A43" t="s">
+        <v>100</v>
+      </c>
+      <c r="B43">
+        <v>69.900000000000006</v>
+      </c>
+      <c r="C43">
+        <v>67.3</v>
+      </c>
+      <c r="D43">
+        <v>79</v>
+      </c>
+      <c r="E43">
+        <v>74.2</v>
+      </c>
+      <c r="F43">
+        <v>40.5</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A44" t="s">
+        <v>101</v>
+      </c>
+      <c r="B44">
+        <v>69.2</v>
+      </c>
+      <c r="C44">
+        <v>69.2</v>
+      </c>
+      <c r="D44">
+        <v>76.599999999999994</v>
+      </c>
+      <c r="E44">
+        <v>76.099999999999994</v>
+      </c>
+      <c r="F44">
+        <v>38.700000000000003</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
+        <v>102</v>
+      </c>
+      <c r="B45">
+        <v>61.8</v>
+      </c>
+      <c r="C45">
+        <v>63</v>
+      </c>
+      <c r="D45">
+        <v>65.599999999999994</v>
+      </c>
+      <c r="E45">
+        <v>63.4</v>
+      </c>
+      <c r="F45">
+        <v>39.200000000000003</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A46" t="s">
+        <v>103</v>
+      </c>
+      <c r="B46">
+        <v>71.5</v>
+      </c>
+      <c r="C46">
+        <v>68.099999999999994</v>
+      </c>
+      <c r="D46">
+        <v>87</v>
+      </c>
+      <c r="E46">
+        <v>82.7</v>
+      </c>
+      <c r="F46">
+        <v>39.200000000000003</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
+        <v>104</v>
+      </c>
+      <c r="B47">
+        <v>77.5</v>
+      </c>
+      <c r="C47">
+        <v>77.900000000000006</v>
+      </c>
+      <c r="D47">
+        <v>70.8</v>
+      </c>
+      <c r="E47">
+        <v>75.5</v>
+      </c>
+      <c r="F47">
+        <v>38.299999999999997</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A48" t="s">
+        <v>105</v>
+      </c>
+      <c r="B48">
+        <v>80.599999999999994</v>
+      </c>
+      <c r="C48">
+        <v>82.9</v>
+      </c>
+      <c r="D48">
+        <v>73.3</v>
+      </c>
+      <c r="E48">
+        <v>82.5</v>
+      </c>
+      <c r="F48">
+        <v>38.9</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
+        <v>106</v>
+      </c>
+      <c r="B49">
+        <v>76.8</v>
+      </c>
+      <c r="C49">
+        <v>78.099999999999994</v>
+      </c>
+      <c r="D49">
+        <v>78.400000000000006</v>
+      </c>
+      <c r="E49">
+        <v>76.599999999999994</v>
+      </c>
+      <c r="F49">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
+        <v>107</v>
+      </c>
+      <c r="B50">
+        <v>83</v>
+      </c>
+      <c r="C50">
+        <v>83.1</v>
+      </c>
+      <c r="D50">
+        <v>82.7</v>
+      </c>
+      <c r="E50">
+        <v>77.099999999999994</v>
+      </c>
+      <c r="F50">
+        <v>40.700000000000003</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A51" t="s">
+        <v>108</v>
+      </c>
+      <c r="B51">
+        <v>78.3</v>
+      </c>
+      <c r="C51">
+        <v>81.2</v>
+      </c>
+      <c r="D51">
+        <v>70.7</v>
+      </c>
+      <c r="E51">
+        <v>74.5</v>
+      </c>
+      <c r="F51">
+        <v>40.799999999999997</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A52" t="s">
+        <v>109</v>
+      </c>
+      <c r="B52">
+        <v>71.7</v>
+      </c>
+      <c r="C52">
+        <v>74.7</v>
+      </c>
+      <c r="D52">
+        <v>65.5</v>
+      </c>
+      <c r="E52">
+        <v>63.1</v>
+      </c>
+      <c r="F52">
+        <v>40.799999999999997</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A53" t="s">
+        <v>110</v>
+      </c>
+      <c r="B53">
+        <v>86.8</v>
+      </c>
+      <c r="C53">
+        <v>91</v>
+      </c>
+      <c r="D53">
+        <v>66.2</v>
+      </c>
+      <c r="E53">
+        <v>76.400000000000006</v>
+      </c>
+      <c r="F53">
+        <v>39.1</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A54" t="s">
+        <v>111</v>
+      </c>
+      <c r="B54">
+        <v>61.1</v>
+      </c>
+      <c r="C54">
+        <v>61</v>
+      </c>
+      <c r="D54">
+        <v>61.7</v>
+      </c>
+      <c r="E54">
+        <v>59.3</v>
+      </c>
+      <c r="F54">
+        <v>39.200000000000003</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A55" t="s">
+        <v>112</v>
+      </c>
+      <c r="B55">
+        <v>87</v>
+      </c>
+      <c r="C55">
+        <v>87.4</v>
+      </c>
+      <c r="D55">
+        <v>85.6</v>
+      </c>
+      <c r="E55">
+        <v>89.6</v>
+      </c>
+      <c r="F55">
+        <v>41.5</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A56" t="s">
+        <v>113</v>
+      </c>
+      <c r="B56">
+        <v>85.1</v>
+      </c>
+      <c r="C56">
+        <v>84.5</v>
+      </c>
+      <c r="D56">
+        <v>83.3</v>
+      </c>
+      <c r="E56">
+        <v>81</v>
+      </c>
+      <c r="F56">
+        <v>40.200000000000003</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A57" t="s">
+        <v>114</v>
+      </c>
+      <c r="B57">
+        <v>74.2</v>
+      </c>
+      <c r="C57">
+        <v>75.599999999999994</v>
+      </c>
+      <c r="D57">
+        <v>86.4</v>
+      </c>
+      <c r="E57">
+        <v>86.7</v>
+      </c>
+      <c r="F57">
+        <v>39.5</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A58" t="s">
+        <v>115</v>
+      </c>
+      <c r="B58">
+        <v>88.1</v>
+      </c>
+      <c r="C58">
+        <v>88.3</v>
+      </c>
+      <c r="D58">
+        <v>73.8</v>
+      </c>
+      <c r="E58">
+        <v>76.8</v>
+      </c>
+      <c r="F58">
+        <v>39.4</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A59" t="s">
+        <v>116</v>
+      </c>
+      <c r="B59">
+        <v>61.7</v>
+      </c>
+      <c r="C59">
+        <v>60</v>
+      </c>
+      <c r="D59">
+        <v>71.599999999999994</v>
+      </c>
+      <c r="E59">
+        <v>73.3</v>
+      </c>
+      <c r="F59">
+        <v>43.8</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A60" t="s">
+        <v>117</v>
+      </c>
+      <c r="B60">
+        <v>69.5</v>
+      </c>
+      <c r="C60">
+        <v>71.099999999999994</v>
+      </c>
+      <c r="D60">
+        <v>80.5</v>
+      </c>
+      <c r="E60">
+        <v>75.7</v>
+      </c>
+      <c r="F60">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A61" t="s">
+        <v>118</v>
+      </c>
+      <c r="B61">
+        <v>65.400000000000006</v>
+      </c>
+      <c r="C61">
+        <v>62.6</v>
+      </c>
+      <c r="D61">
+        <v>71</v>
+      </c>
+      <c r="E61">
+        <v>66.599999999999994</v>
+      </c>
+      <c r="F61">
+        <v>39.700000000000003</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A62" t="s">
+        <v>119</v>
+      </c>
+      <c r="B62">
+        <v>56.5</v>
+      </c>
+      <c r="C62">
+        <v>60</v>
+      </c>
+      <c r="D62">
+        <v>55.2</v>
+      </c>
+      <c r="E62">
+        <v>62.4</v>
+      </c>
+      <c r="F62">
+        <v>39.1</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A63" t="s">
+        <v>120</v>
+      </c>
+      <c r="B63">
+        <v>83.7</v>
+      </c>
+      <c r="C63">
+        <v>88.4</v>
+      </c>
+      <c r="D63">
+        <v>67.3</v>
+      </c>
+      <c r="E63">
+        <v>76.900000000000006</v>
+      </c>
+      <c r="F63">
+        <v>39.9</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A64" t="s">
+        <v>121</v>
+      </c>
+      <c r="B64">
+        <v>69.8</v>
+      </c>
+      <c r="C64">
+        <v>66.599999999999994</v>
+      </c>
+      <c r="D64">
+        <v>81.599999999999994</v>
+      </c>
+      <c r="E64">
+        <v>81.3</v>
+      </c>
+      <c r="F64">
+        <v>40.200000000000003</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A65" t="s">
+        <v>122</v>
+      </c>
+      <c r="B65">
+        <v>83</v>
+      </c>
+      <c r="C65">
+        <v>83.3</v>
+      </c>
+      <c r="D65">
+        <v>81.599999999999994</v>
+      </c>
+      <c r="E65">
+        <v>86.6</v>
+      </c>
+      <c r="F65">
+        <v>40.1</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A66" t="s">
+        <v>123</v>
+      </c>
+      <c r="B66">
+        <v>86.9</v>
+      </c>
+      <c r="C66">
+        <v>85.7</v>
+      </c>
+      <c r="D66">
+        <v>83.1</v>
+      </c>
+      <c r="E66">
+        <v>83.4</v>
+      </c>
+      <c r="F66">
+        <v>42.1</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A67" t="s">
+        <v>124</v>
+      </c>
+      <c r="B67">
+        <v>85.8</v>
+      </c>
+      <c r="C67">
+        <v>83.9</v>
+      </c>
+      <c r="D67">
+        <v>77.2</v>
+      </c>
+      <c r="E67">
+        <v>76.099999999999994</v>
+      </c>
+      <c r="F67">
+        <v>38.4</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A68" t="s">
+        <v>125</v>
+      </c>
+      <c r="B68">
+        <v>80.7</v>
+      </c>
+      <c r="C68">
+        <v>78.099999999999994</v>
+      </c>
+      <c r="D68">
+        <v>83.5</v>
+      </c>
+      <c r="E68">
+        <v>80.5</v>
+      </c>
+      <c r="F68">
+        <v>41.2</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A69" t="s">
+        <v>126</v>
+      </c>
+      <c r="B69">
+        <v>78</v>
+      </c>
+      <c r="C69">
+        <v>78.599999999999994</v>
+      </c>
+      <c r="D69">
+        <v>68.3</v>
+      </c>
+      <c r="E69">
+        <v>72.400000000000006</v>
+      </c>
+      <c r="F69">
+        <v>40.200000000000003</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A70" t="s">
+        <v>127</v>
+      </c>
+      <c r="B70">
+        <v>69.400000000000006</v>
+      </c>
+      <c r="C70">
+        <v>71.5</v>
+      </c>
+      <c r="D70">
+        <v>62.8</v>
+      </c>
+      <c r="E70">
+        <v>56.7</v>
+      </c>
+      <c r="F70">
+        <v>38.700000000000003</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A71" t="s">
+        <v>128</v>
+      </c>
+      <c r="B71">
+        <v>74.2</v>
+      </c>
+      <c r="C71">
+        <v>70.5</v>
+      </c>
+      <c r="D71">
+        <v>89.1</v>
+      </c>
+      <c r="E71">
+        <v>85</v>
+      </c>
+      <c r="F71">
+        <v>40.299999999999997</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A72" t="s">
+        <v>129</v>
+      </c>
+      <c r="B72">
+        <v>76.3</v>
+      </c>
+      <c r="C72">
+        <v>76.3</v>
+      </c>
+      <c r="D72">
+        <v>70.400000000000006</v>
+      </c>
+      <c r="E72">
+        <v>75</v>
+      </c>
+      <c r="F72">
+        <v>40.299999999999997</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A73" t="s">
+        <v>130</v>
+      </c>
+      <c r="B73">
+        <v>88.8</v>
+      </c>
+      <c r="C73">
+        <v>86.4</v>
+      </c>
+      <c r="D73">
+        <v>87.9</v>
+      </c>
+      <c r="E73">
+        <v>91.8</v>
+      </c>
+      <c r="F73">
+        <v>37.4</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A74" t="s">
+        <v>131</v>
+      </c>
+      <c r="B74">
+        <v>74.400000000000006</v>
+      </c>
+      <c r="C74">
+        <v>72.599999999999994</v>
+      </c>
+      <c r="D74">
+        <v>85.6</v>
+      </c>
+      <c r="E74">
+        <v>84.7</v>
+      </c>
+      <c r="F74">
+        <v>43.6</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A75" t="s">
+        <v>132</v>
+      </c>
+      <c r="B75">
+        <v>77.5</v>
+      </c>
+      <c r="C75">
+        <v>74.8</v>
+      </c>
+      <c r="D75">
+        <v>84.1</v>
+      </c>
+      <c r="E75">
+        <v>82.5</v>
+      </c>
+      <c r="F75">
+        <v>37.5</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A76" t="s">
+        <v>133</v>
+      </c>
+      <c r="B76">
+        <v>72</v>
+      </c>
+      <c r="C76">
+        <v>76.099999999999994</v>
+      </c>
+      <c r="D76">
+        <v>68</v>
+      </c>
+      <c r="E76">
+        <v>67</v>
+      </c>
+      <c r="F76">
+        <v>42.8</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A77" t="s">
+        <v>134</v>
+      </c>
+      <c r="B77">
+        <v>73.400000000000006</v>
+      </c>
+      <c r="C77">
+        <v>73.599999999999994</v>
+      </c>
+      <c r="D77">
+        <v>74.599999999999994</v>
+      </c>
+      <c r="E77">
+        <v>71.599999999999994</v>
+      </c>
+      <c r="F77">
+        <v>38.700000000000003</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A78" t="s">
+        <v>135</v>
+      </c>
+      <c r="B78">
+        <v>74.099999999999994</v>
+      </c>
+      <c r="C78">
+        <v>71.599999999999994</v>
+      </c>
+      <c r="D78">
+        <v>82.6</v>
+      </c>
+      <c r="E78">
+        <v>80.599999999999994</v>
+      </c>
+      <c r="F78">
+        <v>37.700000000000003</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A79" t="s">
+        <v>136</v>
+      </c>
+      <c r="B79">
+        <v>72</v>
+      </c>
+      <c r="C79">
+        <v>68.400000000000006</v>
+      </c>
+      <c r="D79">
+        <v>76.3</v>
+      </c>
+      <c r="E79">
+        <v>71.099999999999994</v>
+      </c>
+      <c r="F79">
+        <v>43.4</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A80" t="s">
+        <v>137</v>
+      </c>
+      <c r="B80">
+        <v>70.900000000000006</v>
+      </c>
+      <c r="C80">
+        <v>75</v>
+      </c>
+      <c r="D80">
+        <v>63</v>
+      </c>
+      <c r="E80">
+        <v>61.1</v>
+      </c>
+      <c r="F80">
+        <v>43.8</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A81" t="s">
+        <v>138</v>
+      </c>
+      <c r="B81">
+        <v>74</v>
+      </c>
+      <c r="C81">
+        <v>70.400000000000006</v>
+      </c>
+      <c r="D81">
+        <v>88.1</v>
+      </c>
+      <c r="E81">
+        <v>89.7</v>
+      </c>
+      <c r="F81">
+        <v>39.799999999999997</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A82" t="s">
+        <v>139</v>
+      </c>
+      <c r="B82">
+        <v>80.8</v>
+      </c>
+      <c r="C82">
+        <v>78.2</v>
+      </c>
+      <c r="D82">
+        <v>78.400000000000006</v>
+      </c>
+      <c r="E82">
+        <v>76.400000000000006</v>
+      </c>
+      <c r="F82">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A83" t="s">
+        <v>140</v>
+      </c>
+      <c r="B83">
+        <v>63.9</v>
+      </c>
+      <c r="C83">
+        <v>64.900000000000006</v>
+      </c>
+      <c r="D83">
+        <v>70.3</v>
+      </c>
+      <c r="E83">
+        <v>63.6</v>
+      </c>
+      <c r="F83">
+        <v>36.799999999999997</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A84" t="s">
+        <v>141</v>
+      </c>
+      <c r="B84">
+        <v>76.8</v>
+      </c>
+      <c r="C84">
+        <v>80</v>
+      </c>
+      <c r="D84">
+        <v>71</v>
+      </c>
+      <c r="E84">
+        <v>74.400000000000006</v>
+      </c>
+      <c r="F84">
+        <v>41.6</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A85" t="s">
+        <v>142</v>
+      </c>
+      <c r="B85">
+        <v>86.2</v>
+      </c>
+      <c r="C85">
+        <v>88.6</v>
+      </c>
+      <c r="D85">
+        <v>71.3</v>
+      </c>
+      <c r="E85">
+        <v>75.7</v>
+      </c>
+      <c r="F85">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A86" t="s">
+        <v>143</v>
+      </c>
+      <c r="B86">
+        <v>85.7</v>
+      </c>
+      <c r="C86">
+        <v>82.4</v>
+      </c>
+      <c r="D86">
+        <v>87.7</v>
+      </c>
+      <c r="E86">
+        <v>88.5</v>
+      </c>
+      <c r="F86">
+        <v>41.4</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A87" t="s">
+        <v>144</v>
+      </c>
+      <c r="B87">
+        <v>74.7</v>
+      </c>
+      <c r="C87">
+        <v>73.599999999999994</v>
+      </c>
+      <c r="D87">
+        <v>87.6</v>
+      </c>
+      <c r="E87">
+        <v>83.8</v>
+      </c>
+      <c r="F87">
+        <v>39.9</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A88" t="s">
+        <v>145</v>
+      </c>
+      <c r="B88">
+        <v>74.7</v>
+      </c>
+      <c r="C88">
+        <v>72.400000000000006</v>
+      </c>
+      <c r="D88">
+        <v>87.6</v>
+      </c>
+      <c r="E88">
+        <v>84</v>
+      </c>
+      <c r="F88">
+        <v>38.700000000000003</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A89" t="s">
+        <v>146</v>
+      </c>
+      <c r="B89">
+        <v>84.9</v>
+      </c>
+      <c r="C89">
+        <v>83.9</v>
+      </c>
+      <c r="D89">
+        <v>89.5</v>
+      </c>
+      <c r="E89">
+        <v>89.2</v>
+      </c>
+      <c r="F89">
+        <v>41.4</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A90" t="s">
+        <v>147</v>
+      </c>
+      <c r="B90">
+        <v>66.900000000000006</v>
+      </c>
+      <c r="C90">
+        <v>70.5</v>
+      </c>
+      <c r="D90">
+        <v>66</v>
+      </c>
+      <c r="E90">
+        <v>61.7</v>
+      </c>
+      <c r="F90">
+        <v>42.2</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A91" t="s">
+        <v>148</v>
+      </c>
+      <c r="B91">
+        <v>76.8</v>
+      </c>
+      <c r="C91">
+        <v>74.599999999999994</v>
+      </c>
+      <c r="D91">
+        <v>77.3</v>
+      </c>
+      <c r="E91">
+        <v>72.099999999999994</v>
+      </c>
+      <c r="F91">
+        <v>40.200000000000003</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A92" t="s">
+        <v>149</v>
+      </c>
+      <c r="B92">
+        <v>88.4</v>
+      </c>
+      <c r="C92">
+        <v>87.4</v>
+      </c>
+      <c r="D92">
+        <v>84.4</v>
+      </c>
+      <c r="E92">
+        <v>89.3</v>
+      </c>
+      <c r="F92">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A93" t="s">
+        <v>150</v>
+      </c>
+      <c r="B93">
+        <v>68.7</v>
+      </c>
+      <c r="C93">
+        <v>72.3</v>
+      </c>
+      <c r="D93">
+        <v>63.1</v>
+      </c>
+      <c r="E93">
+        <v>57.8</v>
+      </c>
+      <c r="F93">
+        <v>39.200000000000003</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A94" t="s">
+        <v>151</v>
+      </c>
+      <c r="B94">
+        <v>70.3</v>
+      </c>
+      <c r="C94">
+        <v>67.7</v>
+      </c>
+      <c r="D94">
+        <v>79.400000000000006</v>
+      </c>
+      <c r="E94">
+        <v>80.2</v>
+      </c>
+      <c r="F94">
+        <v>40.700000000000003</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A95" t="s">
+        <v>152</v>
+      </c>
+      <c r="B95">
+        <v>73.599999999999994</v>
+      </c>
+      <c r="C95">
+        <v>74</v>
+      </c>
+      <c r="D95">
+        <v>70.8</v>
+      </c>
+      <c r="E95">
+        <v>69.900000000000006</v>
+      </c>
+      <c r="F95">
+        <v>41.9</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A96" t="s">
+        <v>153</v>
+      </c>
+      <c r="B96">
+        <v>83.7</v>
+      </c>
+      <c r="C96">
+        <v>81.5</v>
+      </c>
+      <c r="D96">
+        <v>88.6</v>
+      </c>
+      <c r="E96">
+        <v>87.9</v>
+      </c>
+      <c r="F96">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A97" t="s">
+        <v>154</v>
+      </c>
+      <c r="B97">
+        <v>79.400000000000006</v>
+      </c>
+      <c r="C97">
+        <v>80.8</v>
+      </c>
+      <c r="D97">
+        <v>67.5</v>
+      </c>
+      <c r="E97">
+        <v>69.5</v>
+      </c>
+      <c r="F97">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A98" t="s">
+        <v>155</v>
+      </c>
+      <c r="B98">
+        <v>81.2</v>
+      </c>
+      <c r="C98">
+        <v>84.8</v>
+      </c>
+      <c r="D98">
+        <v>64.8</v>
+      </c>
+      <c r="E98">
+        <v>71.099999999999994</v>
+      </c>
+      <c r="F98">
+        <v>40.299999999999997</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A99" t="s">
+        <v>156</v>
+      </c>
+      <c r="B99">
+        <v>72.8</v>
+      </c>
+      <c r="C99">
+        <v>73.599999999999994</v>
+      </c>
+      <c r="D99">
+        <v>76.900000000000006</v>
+      </c>
+      <c r="E99">
+        <v>75.099999999999994</v>
+      </c>
+      <c r="F99">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A100" t="s">
+        <v>157</v>
+      </c>
+      <c r="B100">
+        <v>89.6</v>
+      </c>
+      <c r="C100">
+        <v>88.7</v>
+      </c>
+      <c r="D100">
+        <v>83.5</v>
+      </c>
+      <c r="E100">
+        <v>86.3</v>
+      </c>
+      <c r="F100">
+        <v>40.799999999999997</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A101" t="s">
+        <v>158</v>
+      </c>
+      <c r="B101">
+        <v>74.3</v>
+      </c>
+      <c r="C101">
+        <v>73.099999999999994</v>
+      </c>
+      <c r="D101">
+        <v>84.7</v>
+      </c>
+      <c r="E101">
+        <v>86.1</v>
+      </c>
+      <c r="F101">
+        <v>39.299999999999997</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>